<commit_message>
Add manual ASSURANCE/TAXES section to bat recap sheets
Always append Assurance / Taxe foncière / Autres taxes rows at end of
Récap BAT sheets (not site recap) so amounts can be filled manually.
Each poste has a detail row + sous-total, styled like the rest of the recap.

https://claude.ai/code/session_016DCHgeFEbekAwEc4Sro4Qi
</commit_message>
<xml_diff>
--- a/regularisation_MEAUX_PN01_2025.xlsx
+++ b/regularisation_MEAUX_PN01_2025.xlsx
@@ -1465,7 +1465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1988,7 +1988,7 @@
       </c>
     </row>
     <row r="29" ht="6" customHeight="1"/>
-    <row r="30" ht="25.55" customHeight="1">
+    <row r="30" ht="6" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
           <t>TOTAL GÉNÉRAL — CHARGES RÉCUPÉRABLES</t>
@@ -1999,12 +1999,104 @@
         <v/>
       </c>
     </row>
+    <row r="31" ht="21.75" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>── ASSURANCE / TAXES ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Assurance</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15.05" customHeight="1">
+      <c r="A33" s="6" t="inlineStr"/>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+    </row>
+    <row r="34" ht="15.8" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sous-total — Assurance</t>
+        </is>
+      </c>
+      <c r="E34" s="10">
+        <f>E33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Taxe foncière</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15.05" customHeight="1">
+      <c r="A36" s="6" t="inlineStr"/>
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
+    </row>
+    <row r="37" ht="15.8" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sous-total — Taxe foncière</t>
+        </is>
+      </c>
+      <c r="E37" s="10">
+        <f>E36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Autres taxes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15.05" customHeight="1">
+      <c r="A39" s="6" t="inlineStr"/>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="n"/>
+    </row>
+    <row r="40" ht="15.8" customHeight="1">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sous-total — Autres taxes</t>
+        </is>
+      </c>
+      <c r="E40" s="10">
+        <f>E39</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A34:D34"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="A21:D21"/>
@@ -2024,7 +2116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5601,7 +5693,7 @@
       </c>
     </row>
     <row r="157" ht="6" customHeight="1"/>
-    <row r="158" ht="25.55" customHeight="1">
+    <row r="158" ht="6" customHeight="1">
       <c r="A158" s="13" t="inlineStr">
         <is>
           <t>TOTAL GÉNÉRAL — CHARGES RÉCUPÉRABLES</t>
@@ -5612,11 +5704,101 @@
         <v/>
       </c>
     </row>
+    <row r="159" ht="21.75" customHeight="1">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>── ASSURANCE / TAXES ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Assurance</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="15.05" customHeight="1">
+      <c r="A161" s="6" t="inlineStr"/>
+      <c r="B161" s="11" t="n"/>
+      <c r="C161" s="11" t="n"/>
+      <c r="D161" s="11" t="n"/>
+      <c r="E161" s="8" t="n"/>
+      <c r="F161" s="8" t="n"/>
+      <c r="G161" s="8" t="n"/>
+    </row>
+    <row r="162" ht="15.8" customHeight="1">
+      <c r="A162" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sous-total — Assurance</t>
+        </is>
+      </c>
+      <c r="E162" s="10">
+        <f>E161</f>
+        <v/>
+      </c>
+    </row>
+    <row r="163" ht="18" customHeight="1">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Taxe foncière</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="15.05" customHeight="1">
+      <c r="A164" s="6" t="inlineStr"/>
+      <c r="B164" s="11" t="n"/>
+      <c r="C164" s="11" t="n"/>
+      <c r="D164" s="11" t="n"/>
+      <c r="E164" s="8" t="n"/>
+      <c r="F164" s="8" t="n"/>
+      <c r="G164" s="8" t="n"/>
+    </row>
+    <row r="165" ht="15.8" customHeight="1">
+      <c r="A165" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sous-total — Taxe foncière</t>
+        </is>
+      </c>
+      <c r="E165" s="10">
+        <f>E164</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166" ht="18" customHeight="1">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Autres taxes</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="15.05" customHeight="1">
+      <c r="A167" s="6" t="inlineStr"/>
+      <c r="B167" s="11" t="n"/>
+      <c r="C167" s="11" t="n"/>
+      <c r="D167" s="11" t="n"/>
+      <c r="E167" s="8" t="n"/>
+      <c r="F167" s="8" t="n"/>
+      <c r="G167" s="8" t="n"/>
+    </row>
+    <row r="168" ht="15.8" customHeight="1">
+      <c r="A168" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Sous-total — Autres taxes</t>
+        </is>
+      </c>
+      <c r="E168" s="10">
+        <f>E167</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="37">
+    <mergeCell ref="A159:G159"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A96:D96"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A165:D165"/>
     <mergeCell ref="A81:D81"/>
     <mergeCell ref="A156:D156"/>
     <mergeCell ref="A63:D63"/>
@@ -5631,7 +5813,9 @@
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A132:D132"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A168:D168"/>
     <mergeCell ref="A119:D119"/>
+    <mergeCell ref="A162:D162"/>
     <mergeCell ref="A87:D87"/>
     <mergeCell ref="A41:G41"/>
     <mergeCell ref="A128:G128"/>

</xml_diff>